<commit_message>
Release v1.0.4: hidden sheets no longer need a password, document how to save a record
</commit_message>
<xml_diff>
--- a/Business Finance Pro v1.0.3.xlsx
+++ b/Business Finance Pro v1.0.3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saad\BusinessFinancePro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08D99F9-2ECF-4E80-A232-3445F91A2CF4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C419FA-B157-47C4-BE66-9B6F917DCEB5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8235" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="1" r:id="rId1"/>
@@ -1713,43 +1713,44 @@
     <xf numFmtId="169" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1761,6 +1762,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1775,15 +1782,12 @@
     <xf numFmtId="169" fontId="10" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1792,11 +1796,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1811,13 +1814,10 @@
     <xf numFmtId="166" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1835,13 +1835,13 @@
   </cellStyles>
   <dxfs count="46">
     <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;Rs &quot;#,##0.00"/>
+      <numFmt numFmtId="170" formatCode="&quot;Rs &quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="174" formatCode="&quot;€&quot;#,##0.00"/>
+      <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="173" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="172" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <font>
@@ -1892,13 +1892,13 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;Rs &quot;#,##0.00"/>
+      <numFmt numFmtId="170" formatCode="&quot;Rs &quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="174" formatCode="&quot;€&quot;#,##0.00"/>
+      <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="173" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="172" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <font>
@@ -1981,13 +1981,13 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;Rs &quot;#,##0.00"/>
+      <numFmt numFmtId="170" formatCode="&quot;Rs &quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="174" formatCode="&quot;€&quot;#,##0.00"/>
+      <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="173" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="172" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <font>
@@ -2070,22 +2070,22 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="175" formatCode="&quot;Rs &quot;#,##0.00"/>
+      <numFmt numFmtId="170" formatCode="&quot;Rs &quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="174" formatCode="&quot;€&quot;#,##0.00"/>
+      <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="173" formatCode="&quot;£&quot;#,##0.00"/>
+      <numFmt numFmtId="172" formatCode="&quot;£&quot;#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="172" formatCode="&quot;Rs &quot;#,##0"/>
+      <numFmt numFmtId="173" formatCode="&quot;Rs &quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="171" formatCode="&quot;€&quot;#,##0"/>
+      <numFmt numFmtId="174" formatCode="&quot;€&quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="170" formatCode="&quot;£&quot;#,##0"/>
+      <numFmt numFmtId="175" formatCode="&quot;£&quot;#,##0"/>
     </dxf>
     <dxf>
       <font>
@@ -2583,12 +2583,12 @@
     </row>
     <row r="2" spans="1:14" ht="39.75" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="56" t="str">
+      <c r="B2" s="46" t="str">
         <f>CurrentBusinessName</f>
         <v>Riverside Design Studio</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="3" t="s">
         <v>0</v>
@@ -2630,7 +2630,7 @@
     </row>
     <row r="4" spans="1:14" ht="19.5" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="44"/>
@@ -2664,7 +2664,7 @@
     </row>
     <row r="6" spans="1:14" ht="19.5" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="54" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="44"/>
@@ -2682,7 +2682,7 @@
     </row>
     <row r="7" spans="1:14" ht="55.5" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="50" t="str">
+      <c r="B7" s="57" t="str">
         <f ca="1">calcHealthTitle</f>
         <v>Excellent</v>
       </c>
@@ -2701,7 +2701,7 @@
     </row>
     <row r="8" spans="1:14" ht="18" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="46" t="str">
+      <c r="B8" s="54" t="str">
         <f ca="1">calcHealthSubtitle</f>
         <v>Income is well ahead of spending this month</v>
       </c>
@@ -2736,13 +2736,13 @@
     </row>
     <row r="10" spans="1:14" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="56" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="43" t="s">
+      <c r="F10" s="56" t="s">
         <v>8</v>
       </c>
       <c r="G10" s="44"/>
@@ -2778,11 +2778,11 @@
     </row>
     <row r="12" spans="1:14" ht="18" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="54"/>
+      <c r="B12" s="55"/>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="54"/>
+      <c r="F12" s="55"/>
       <c r="G12" s="44"/>
       <c r="H12" s="44"/>
       <c r="I12" s="1"/>
@@ -2826,20 +2826,20 @@
     </row>
     <row r="15" spans="1:14" ht="19.5" customHeight="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="48"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="52"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="52"/>
+      <c r="L15" s="52"/>
+      <c r="M15" s="53"/>
       <c r="N15" s="1"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1">
@@ -2986,25 +2986,25 @@
     </row>
     <row r="23" spans="1:14" ht="19.5" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="47" t="s">
+      <c r="B23" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48"/>
-      <c r="J23" s="48"/>
-      <c r="K23" s="48"/>
-      <c r="L23" s="48"/>
-      <c r="M23" s="49"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="52"/>
+      <c r="E23" s="52"/>
+      <c r="F23" s="52"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="52"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="52"/>
+      <c r="M23" s="53"/>
       <c r="N23" s="1"/>
     </row>
     <row r="24" spans="1:14" ht="18" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="51" t="str">
+      <c r="B24" s="48" t="str">
         <f ca="1">_xlfn.TEXTJOIN(" ",TRUE(),InsightItem1Message,InsightItem2Message,InsightItem3Message)</f>
         <v>Your biggest expense this month was Supplies at $165. You paid City Wholesale Supplies more than anyone else this month, totaling $165. You've brought in $850 so far this month.</v>
       </c>
@@ -3018,12 +3018,12 @@
       <c r="J24" s="44"/>
       <c r="K24" s="44"/>
       <c r="L24" s="44"/>
-      <c r="M24" s="52"/>
+      <c r="M24" s="49"/>
       <c r="N24" s="1"/>
     </row>
     <row r="25" spans="1:14" ht="18" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="53"/>
+      <c r="B25" s="50"/>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
@@ -3034,12 +3034,12 @@
       <c r="J25" s="44"/>
       <c r="K25" s="44"/>
       <c r="L25" s="44"/>
-      <c r="M25" s="52"/>
+      <c r="M25" s="49"/>
       <c r="N25" s="1"/>
     </row>
     <row r="26" spans="1:14" ht="18" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="53"/>
+      <c r="B26" s="50"/>
       <c r="C26" s="44"/>
       <c r="D26" s="44"/>
       <c r="E26" s="44"/>
@@ -3050,7 +3050,7 @@
       <c r="J26" s="44"/>
       <c r="K26" s="44"/>
       <c r="L26" s="44"/>
-      <c r="M26" s="52"/>
+      <c r="M26" s="49"/>
       <c r="N26" s="1"/>
     </row>
     <row r="27" spans="1:14" ht="15.75" customHeight="1">
@@ -6011,11 +6011,11 @@
     </row>
     <row r="2" spans="1:14" ht="39.75" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
         <v>0</v>
@@ -6057,7 +6057,7 @@
     </row>
     <row r="4" spans="1:14" ht="19.5" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="44"/>
@@ -6091,138 +6091,138 @@
     </row>
     <row r="6" spans="1:14" ht="19.5" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="53"/>
       <c r="N6" s="1"/>
     </row>
     <row r="7" spans="1:14" ht="21.75" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="60" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
       <c r="E7" s="10"/>
-      <c r="F7" s="60" t="s">
+      <c r="F7" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
-      <c r="L7" s="61"/>
-      <c r="M7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="63"/>
       <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:14" ht="21.75" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="60" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
       <c r="E8" s="10"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="62"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="62"/>
+      <c r="K8" s="62"/>
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
       <c r="N8" s="1"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="60" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="60" t="s">
+      <c r="F9" s="61" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="61"/>
-      <c r="H9" s="61"/>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+      <c r="L9" s="62"/>
+      <c r="M9" s="63"/>
       <c r="N9" s="1"/>
     </row>
     <row r="10" spans="1:14" ht="21.75" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="60" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
       <c r="E10" s="10"/>
-      <c r="F10" s="60" t="s">
+      <c r="F10" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="63"/>
       <c r="N10" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="21.75" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="58" t="s">
+      <c r="B11" s="60" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="60" t="s">
+      <c r="F11" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
-      <c r="J11" s="61"/>
-      <c r="K11" s="61"/>
-      <c r="L11" s="61"/>
-      <c r="M11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="62"/>
+      <c r="K11" s="62"/>
+      <c r="L11" s="62"/>
+      <c r="M11" s="63"/>
       <c r="N11" s="1"/>
     </row>
     <row r="12" spans="1:14" ht="21.75" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="67" t="s">
+      <c r="B12" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="63" t="s">
+      <c r="F12" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="64"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="64"/>
-      <c r="K12" s="64"/>
-      <c r="L12" s="64"/>
-      <c r="M12" s="65"/>
+      <c r="G12" s="67"/>
+      <c r="H12" s="67"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="67"/>
+      <c r="K12" s="67"/>
+      <c r="L12" s="67"/>
+      <c r="M12" s="68"/>
       <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1">
@@ -6259,51 +6259,51 @@
     </row>
     <row r="15" spans="1:14" ht="19.5" customHeight="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="48"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48"/>
-      <c r="M15" s="49"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="52"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="52"/>
+      <c r="L15" s="52"/>
+      <c r="M15" s="53"/>
       <c r="N15" s="1"/>
     </row>
     <row r="16" spans="1:14" ht="21.75" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="60" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="44"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="60" t="s">
+      <c r="F16" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="61"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="62"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
+      <c r="I16" s="62"/>
+      <c r="J16" s="62"/>
+      <c r="K16" s="62"/>
+      <c r="L16" s="62"/>
+      <c r="M16" s="63"/>
       <c r="N16" s="1"/>
     </row>
     <row r="17" spans="1:14" ht="21.75" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="60" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="59" t="s">
+      <c r="F17" s="65" t="s">
         <v>28</v>
       </c>
       <c r="G17" s="44"/>
@@ -6312,27 +6312,27 @@
       <c r="J17" s="44"/>
       <c r="K17" s="44"/>
       <c r="L17" s="44"/>
-      <c r="M17" s="52"/>
+      <c r="M17" s="49"/>
       <c r="N17" s="1"/>
     </row>
     <row r="18" spans="1:14" ht="21.75" customHeight="1">
       <c r="A18" s="1"/>
-      <c r="B18" s="67" t="s">
+      <c r="B18" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="63" t="s">
+      <c r="F18" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="64"/>
-      <c r="H18" s="64"/>
-      <c r="I18" s="64"/>
-      <c r="J18" s="64"/>
-      <c r="K18" s="64"/>
-      <c r="L18" s="64"/>
-      <c r="M18" s="65"/>
+      <c r="G18" s="67"/>
+      <c r="H18" s="67"/>
+      <c r="I18" s="67"/>
+      <c r="J18" s="67"/>
+      <c r="K18" s="67"/>
+      <c r="L18" s="67"/>
+      <c r="M18" s="68"/>
       <c r="N18" s="1"/>
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1">
@@ -6369,80 +6369,80 @@
     </row>
     <row r="21" spans="1:14" ht="19.5" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48"/>
-      <c r="H21" s="48"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="48"/>
-      <c r="K21" s="48"/>
-      <c r="L21" s="48"/>
-      <c r="M21" s="49"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="52"/>
+      <c r="J21" s="52"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="52"/>
+      <c r="M21" s="53"/>
       <c r="N21" s="1"/>
     </row>
     <row r="22" spans="1:14" ht="21.75" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="60" t="s">
         <v>32</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="44"/>
       <c r="E22" s="10"/>
-      <c r="F22" s="60" t="s">
+      <c r="F22" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
-      <c r="I22" s="61"/>
-      <c r="J22" s="61"/>
-      <c r="K22" s="61"/>
-      <c r="L22" s="61"/>
-      <c r="M22" s="62"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="62"/>
+      <c r="J22" s="62"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="62"/>
+      <c r="M22" s="63"/>
       <c r="N22" s="1"/>
     </row>
     <row r="23" spans="1:14" ht="21.75" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="60" t="s">
         <v>34</v>
       </c>
       <c r="C23" s="44"/>
       <c r="D23" s="44"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="60" t="s">
+      <c r="F23" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
-      <c r="M23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
+      <c r="M23" s="63"/>
       <c r="N23" s="1"/>
     </row>
     <row r="24" spans="1:14" ht="21.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="67" t="s">
+      <c r="B24" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
       <c r="E24" s="2"/>
-      <c r="F24" s="63" t="s">
+      <c r="F24" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
-      <c r="L24" s="64"/>
-      <c r="M24" s="65"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
+      <c r="L24" s="67"/>
+      <c r="M24" s="68"/>
       <c r="N24" s="1"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" customHeight="1">
@@ -6479,31 +6479,31 @@
     </row>
     <row r="27" spans="1:14" ht="19.5" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48"/>
-      <c r="L27" s="48"/>
-      <c r="M27" s="49"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="52"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="52"/>
+      <c r="L27" s="52"/>
+      <c r="M27" s="53"/>
       <c r="N27" s="1"/>
     </row>
     <row r="28" spans="1:14" ht="21.75" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="58" t="s">
+      <c r="B28" s="60" t="s">
         <v>39</v>
       </c>
       <c r="C28" s="44"/>
       <c r="D28" s="44"/>
       <c r="E28" s="10"/>
-      <c r="F28" s="59" t="str">
+      <c r="F28" s="65" t="str">
         <f>CurrentAppVersion</f>
         <v>1.0.3</v>
       </c>
@@ -6513,18 +6513,18 @@
       <c r="J28" s="44"/>
       <c r="K28" s="44"/>
       <c r="L28" s="44"/>
-      <c r="M28" s="52"/>
+      <c r="M28" s="49"/>
       <c r="N28" s="1"/>
     </row>
     <row r="29" spans="1:14" ht="21.75" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="60" t="s">
         <v>40</v>
       </c>
       <c r="C29" s="44"/>
       <c r="D29" s="44"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="59" t="str">
+      <c r="F29" s="65" t="str">
         <f>CurrentBuildNumber</f>
         <v>2026.10.11-001</v>
       </c>
@@ -6534,18 +6534,18 @@
       <c r="J29" s="44"/>
       <c r="K29" s="44"/>
       <c r="L29" s="44"/>
-      <c r="M29" s="52"/>
+      <c r="M29" s="49"/>
       <c r="N29" s="1"/>
     </row>
     <row r="30" spans="1:14" ht="21.75" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="58" t="s">
+      <c r="B30" s="60" t="s">
         <v>41</v>
       </c>
       <c r="C30" s="44"/>
       <c r="D30" s="44"/>
       <c r="E30" s="10"/>
-      <c r="F30" s="66">
+      <c r="F30" s="69">
         <f>CurrentLastUpdated</f>
         <v>46306</v>
       </c>
@@ -6555,28 +6555,28 @@
       <c r="J30" s="44"/>
       <c r="K30" s="44"/>
       <c r="L30" s="44"/>
-      <c r="M30" s="52"/>
+      <c r="M30" s="49"/>
       <c r="N30" s="1"/>
     </row>
     <row r="31" spans="1:14" ht="21.75" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="67" t="s">
+      <c r="B31" s="64" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="57"/>
-      <c r="D31" s="57"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="68" t="str">
+      <c r="F31" s="58" t="str">
         <f>CurrentLicense</f>
         <v>Licensed to Riverside Design Studio</v>
       </c>
-      <c r="G31" s="57"/>
-      <c r="H31" s="57"/>
-      <c r="I31" s="57"/>
-      <c r="J31" s="57"/>
-      <c r="K31" s="57"/>
-      <c r="L31" s="57"/>
-      <c r="M31" s="69"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="59"/>
       <c r="N31" s="1"/>
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1">
@@ -6614,6 +6614,28 @@
   </sheetData>
   <sheetProtection password="ECAF" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="38">
+    <mergeCell ref="F30:M30"/>
+    <mergeCell ref="F24:M24"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F18:M18"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="F29:M29"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="F11:M11"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F16:M16"/>
+    <mergeCell ref="F10:M10"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F28:M28"/>
+    <mergeCell ref="F22:M22"/>
+    <mergeCell ref="F7:M7"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="F12:M12"/>
+    <mergeCell ref="F8:M8"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="F31:M31"/>
     <mergeCell ref="B4:M4"/>
@@ -6630,28 +6652,6 @@
     <mergeCell ref="F17:M17"/>
     <mergeCell ref="B15:M15"/>
     <mergeCell ref="F23:M23"/>
-    <mergeCell ref="F28:M28"/>
-    <mergeCell ref="F22:M22"/>
-    <mergeCell ref="F7:M7"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F12:M12"/>
-    <mergeCell ref="F30:M30"/>
-    <mergeCell ref="F24:M24"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F18:M18"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="F8:M8"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="F29:M29"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="F11:M11"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F16:M16"/>
-    <mergeCell ref="F10:M10"/>
-    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <dataValidations count="8">
     <dataValidation type="list" sqref="F10" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -7631,12 +7631,12 @@
     </row>
     <row r="2" spans="1:15" ht="18" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="74" t="str">
+      <c r="B2" s="70" t="str">
         <f>CurrentBusinessName</f>
         <v>Riverside Design Studio</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
         <v>0</v>
@@ -7680,7 +7680,7 @@
     </row>
     <row r="4" spans="1:15" ht="27.75" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="44"/>
@@ -7716,168 +7716,168 @@
     </row>
     <row r="6" spans="1:15" ht="23.25" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="53"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="58" t="s">
+      <c r="B7" s="60" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
       <c r="E7" s="10"/>
-      <c r="F7" s="71">
+      <c r="F7" s="72">
         <f ca="1">TODAY()</f>
         <v>46307</v>
       </c>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
-      <c r="L7" s="61"/>
-      <c r="M7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="63"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="60" t="s">
         <v>45</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
       <c r="E8" s="10"/>
-      <c r="F8" s="60" t="s">
+      <c r="F8" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="62"/>
+      <c r="K8" s="62"/>
+      <c r="L8" s="62"/>
+      <c r="M8" s="63"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="60" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="73">
+      <c r="F9" s="71">
         <v>850</v>
       </c>
-      <c r="G9" s="61"/>
-      <c r="H9" s="61"/>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+      <c r="L9" s="62"/>
+      <c r="M9" s="63"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="60" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
       <c r="E10" s="10"/>
-      <c r="F10" s="60" t="s">
+      <c r="F10" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="63"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="58" t="s">
+      <c r="B11" s="60" t="s">
         <v>50</v>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="60" t="s">
+      <c r="F11" s="61" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
-      <c r="J11" s="61"/>
-      <c r="K11" s="61"/>
-      <c r="L11" s="61"/>
-      <c r="M11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="62"/>
+      <c r="K11" s="62"/>
+      <c r="L11" s="62"/>
+      <c r="M11" s="63"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="60" t="s">
         <v>52</v>
       </c>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
       <c r="E12" s="10"/>
-      <c r="F12" s="60" t="s">
+      <c r="F12" s="61" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="61"/>
-      <c r="L12" s="61"/>
-      <c r="M12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="62"/>
+      <c r="L12" s="62"/>
+      <c r="M12" s="63"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="60" t="s">
         <v>54</v>
       </c>
       <c r="C13" s="44"/>
       <c r="D13" s="44"/>
       <c r="E13" s="10"/>
-      <c r="F13" s="60" t="s">
+      <c r="F13" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="61"/>
-      <c r="H13" s="61"/>
-      <c r="I13" s="61"/>
-      <c r="J13" s="61"/>
-      <c r="K13" s="61"/>
-      <c r="L13" s="61"/>
-      <c r="M13" s="62"/>
+      <c r="G13" s="62"/>
+      <c r="H13" s="62"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="62"/>
+      <c r="K13" s="62"/>
+      <c r="L13" s="62"/>
+      <c r="M13" s="63"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
@@ -7917,7 +7917,7 @@
     </row>
     <row r="16" spans="1:15" ht="23.25" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="70" t="str">
+      <c r="B16" s="74" t="str">
         <f>IF(OR(F8="",F9="",F10=""),"Ready to save — fill in the form above first","Ready to save")</f>
         <v>Ready to save</v>
       </c>
@@ -7937,7 +7937,7 @@
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="1"/>
-      <c r="B17" s="72" t="s">
+      <c r="B17" s="73" t="s">
         <v>56</v>
       </c>
       <c r="C17" s="44"/>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="O19" s="36">
         <f ca="1">NOW()</f>
-        <v>46307.087774768515</v>
+        <v>46307.088475694443</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -8067,6 +8067,14 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B17:O17"/>
+    <mergeCell ref="F8:M8"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="F11:M11"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B16:O16"/>
+    <mergeCell ref="F10:M10"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B6:M6"/>
     <mergeCell ref="F13:M13"/>
@@ -8078,14 +8086,6 @@
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="F12:M12"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B17:O17"/>
-    <mergeCell ref="F8:M8"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="F11:M11"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B16:O16"/>
-    <mergeCell ref="F10:M10"/>
-    <mergeCell ref="B13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="E19 F9">
     <cfRule type="expression" dxfId="37" priority="1">
@@ -8174,12 +8174,12 @@
     </row>
     <row r="2" spans="1:15" ht="39.75" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="56" t="str">
+      <c r="B2" s="46" t="str">
         <f>CurrentBusinessName</f>
         <v>Riverside Design Studio</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
         <v>0</v>
@@ -8223,7 +8223,7 @@
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>69</v>
       </c>
       <c r="C4" s="44"/>
@@ -8259,36 +8259,36 @@
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="53"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="75" t="s">
         <v>71</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
       <c r="E7" s="10"/>
-      <c r="F7" s="79" t="s">
+      <c r="F7" s="81" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="44"/>
-      <c r="H7" s="79" t="s">
+      <c r="H7" s="81" t="s">
         <v>72</v>
       </c>
       <c r="I7" s="44"/>
@@ -8297,297 +8297,297 @@
         <v>73</v>
       </c>
       <c r="L7" s="44"/>
-      <c r="M7" s="52"/>
+      <c r="M7" s="49"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="75" t="str">
+      <c r="B8" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],1),tbl_Vendors[VendorID],0)),"")</f>
         <v>City Wholesale Supplies</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
       <c r="E8" s="10"/>
-      <c r="F8" s="76">
+      <c r="F8" s="77">
         <f>IFERROR(INDEX(tbl_Bills[Amount],1),"")</f>
         <v>89</v>
       </c>
       <c r="G8" s="44"/>
-      <c r="H8" s="78">
+      <c r="H8" s="79">
         <f ca="1">IFERROR(INDEX(tbl_Bills[DueDate],1),"")</f>
         <v>46318</v>
       </c>
       <c r="I8" s="44"/>
       <c r="J8" s="44"/>
-      <c r="K8" s="77" t="str">
+      <c r="K8" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],1)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],1)="","",IF(INDEX(tbl_Bills[DueDate],1)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v>Upcoming</v>
       </c>
       <c r="L8" s="44"/>
-      <c r="M8" s="52"/>
+      <c r="M8" s="49"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="75" t="str">
+      <c r="B9" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],2),tbl_Vendors[VendorID],0)),"")</f>
         <v>City Wholesale Supplies</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="76">
+      <c r="F9" s="77">
         <f>IFERROR(INDEX(tbl_Bills[Amount],2),"")</f>
         <v>150</v>
       </c>
       <c r="G9" s="44"/>
-      <c r="H9" s="78">
+      <c r="H9" s="79">
         <f ca="1">IFERROR(INDEX(tbl_Bills[DueDate],2),"")</f>
         <v>46301</v>
       </c>
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
-      <c r="K9" s="77" t="str">
+      <c r="K9" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],2)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],2)="","",IF(INDEX(tbl_Bills[DueDate],2)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v>Overdue</v>
       </c>
       <c r="L9" s="44"/>
-      <c r="M9" s="52"/>
+      <c r="M9" s="49"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="75" t="str">
+      <c r="B10" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],3),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
       <c r="E10" s="10"/>
-      <c r="F10" s="76" t="str">
+      <c r="F10" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],3),"")</f>
         <v/>
       </c>
       <c r="G10" s="44"/>
-      <c r="H10" s="78" t="str">
+      <c r="H10" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],3),"")</f>
         <v/>
       </c>
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
-      <c r="K10" s="77" t="str">
+      <c r="K10" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],3)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],3)="","",IF(INDEX(tbl_Bills[DueDate],3)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L10" s="44"/>
-      <c r="M10" s="52"/>
+      <c r="M10" s="49"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="75" t="str">
+      <c r="B11" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],4),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="76" t="str">
+      <c r="F11" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],4),"")</f>
         <v/>
       </c>
       <c r="G11" s="44"/>
-      <c r="H11" s="78" t="str">
+      <c r="H11" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],4),"")</f>
         <v/>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
-      <c r="K11" s="77" t="str">
+      <c r="K11" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],4)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],4)="","",IF(INDEX(tbl_Bills[DueDate],4)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L11" s="44"/>
-      <c r="M11" s="52"/>
+      <c r="M11" s="49"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="75" t="str">
+      <c r="B12" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],5),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
       <c r="E12" s="10"/>
-      <c r="F12" s="76" t="str">
+      <c r="F12" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],5),"")</f>
         <v/>
       </c>
       <c r="G12" s="44"/>
-      <c r="H12" s="78" t="str">
+      <c r="H12" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],5),"")</f>
         <v/>
       </c>
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
-      <c r="K12" s="77" t="str">
+      <c r="K12" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],5)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],5)="","",IF(INDEX(tbl_Bills[DueDate],5)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L12" s="44"/>
-      <c r="M12" s="52"/>
+      <c r="M12" s="49"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="75" t="str">
+      <c r="B13" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],6),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C13" s="44"/>
       <c r="D13" s="44"/>
       <c r="E13" s="10"/>
-      <c r="F13" s="76" t="str">
+      <c r="F13" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],6),"")</f>
         <v/>
       </c>
       <c r="G13" s="44"/>
-      <c r="H13" s="78" t="str">
+      <c r="H13" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],6),"")</f>
         <v/>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
-      <c r="K13" s="77" t="str">
+      <c r="K13" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],6)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],6)="","",IF(INDEX(tbl_Bills[DueDate],6)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L13" s="44"/>
-      <c r="M13" s="52"/>
+      <c r="M13" s="49"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1">
       <c r="A14" s="1"/>
-      <c r="B14" s="75" t="str">
+      <c r="B14" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],7),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C14" s="44"/>
       <c r="D14" s="44"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="76" t="str">
+      <c r="F14" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],7),"")</f>
         <v/>
       </c>
       <c r="G14" s="44"/>
-      <c r="H14" s="78" t="str">
+      <c r="H14" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],7),"")</f>
         <v/>
       </c>
       <c r="I14" s="44"/>
       <c r="J14" s="44"/>
-      <c r="K14" s="77" t="str">
+      <c r="K14" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],7)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],7)="","",IF(INDEX(tbl_Bills[DueDate],7)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L14" s="44"/>
-      <c r="M14" s="52"/>
+      <c r="M14" s="49"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="75" t="str">
+      <c r="B15" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],8),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C15" s="44"/>
       <c r="D15" s="44"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="76" t="str">
+      <c r="F15" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],8),"")</f>
         <v/>
       </c>
       <c r="G15" s="44"/>
-      <c r="H15" s="78" t="str">
+      <c r="H15" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],8),"")</f>
         <v/>
       </c>
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
-      <c r="K15" s="77" t="str">
+      <c r="K15" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],8)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],8)="","",IF(INDEX(tbl_Bills[DueDate],8)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L15" s="44"/>
-      <c r="M15" s="52"/>
+      <c r="M15" s="49"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="75" t="str">
+      <c r="B16" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],9),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="44"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="76" t="str">
+      <c r="F16" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],9),"")</f>
         <v/>
       </c>
       <c r="G16" s="44"/>
-      <c r="H16" s="78" t="str">
+      <c r="H16" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],9),"")</f>
         <v/>
       </c>
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
-      <c r="K16" s="77" t="str">
+      <c r="K16" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],9)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],9)="","",IF(INDEX(tbl_Bills[DueDate],9)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L16" s="44"/>
-      <c r="M16" s="52"/>
+      <c r="M16" s="49"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" ht="18" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="75" t="str">
+      <c r="B17" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Vendors[VendorName],MATCH(INDEX(tbl_Bills[VendorID],10),tbl_Vendors[VendorID],0)),"")</f>
         <v/>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="76" t="str">
+      <c r="F17" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Bills[Amount],10),"")</f>
         <v/>
       </c>
       <c r="G17" s="44"/>
-      <c r="H17" s="78" t="str">
+      <c r="H17" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Bills[DueDate],10),"")</f>
         <v/>
       </c>
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
-      <c r="K17" s="77" t="str">
+      <c r="K17" s="78" t="str">
         <f ca="1">IFERROR(IF(INDEX(tbl_Bills[Status],10)="Paid","Paid",IF(INDEX(tbl_Bills[DueDate],10)="","",IF(INDEX(tbl_Bills[DueDate],10)&lt;TODAY(),"Overdue","Upcoming"))),"")</f>
         <v/>
       </c>
       <c r="L17" s="44"/>
-      <c r="M17" s="52"/>
+      <c r="M17" s="49"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
@@ -8627,134 +8627,134 @@
     </row>
     <row r="20" spans="1:15" ht="19.5" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48"/>
-      <c r="L20" s="48"/>
-      <c r="M20" s="49"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="52"/>
+      <c r="J20" s="52"/>
+      <c r="K20" s="52"/>
+      <c r="L20" s="52"/>
+      <c r="M20" s="53"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
     <row r="21" spans="1:15" ht="21.75" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="60" t="s">
         <v>71</v>
       </c>
       <c r="C21" s="44"/>
       <c r="D21" s="44"/>
       <c r="E21" s="10"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61"/>
-      <c r="I21" s="61"/>
-      <c r="J21" s="61"/>
-      <c r="K21" s="61"/>
-      <c r="L21" s="61"/>
-      <c r="M21" s="62"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="62"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="63"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
     </row>
     <row r="22" spans="1:15" ht="21.75" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="60" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="44"/>
       <c r="E22" s="10"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
-      <c r="I22" s="61"/>
-      <c r="J22" s="61"/>
-      <c r="K22" s="61"/>
-      <c r="L22" s="61"/>
-      <c r="M22" s="62"/>
+      <c r="F22" s="71"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="62"/>
+      <c r="J22" s="62"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="62"/>
+      <c r="M22" s="63"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="21.75" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="60" t="s">
         <v>72</v>
       </c>
       <c r="C23" s="44"/>
       <c r="D23" s="44"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
-      <c r="M23" s="62"/>
+      <c r="F23" s="72"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
+      <c r="M23" s="63"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="21.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="58" t="s">
+      <c r="B24" s="60" t="s">
         <v>75</v>
       </c>
       <c r="C24" s="44"/>
       <c r="D24" s="44"/>
       <c r="E24" s="10"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
-      <c r="I24" s="61"/>
-      <c r="J24" s="61"/>
-      <c r="K24" s="61"/>
-      <c r="L24" s="61"/>
-      <c r="M24" s="62"/>
+      <c r="F24" s="61"/>
+      <c r="G24" s="62"/>
+      <c r="H24" s="62"/>
+      <c r="I24" s="62"/>
+      <c r="J24" s="62"/>
+      <c r="K24" s="62"/>
+      <c r="L24" s="62"/>
+      <c r="M24" s="63"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="21.75" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="60" t="s">
         <v>76</v>
       </c>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="10"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="61"/>
-      <c r="H25" s="61"/>
-      <c r="I25" s="61"/>
-      <c r="J25" s="61"/>
-      <c r="K25" s="61"/>
-      <c r="L25" s="61"/>
-      <c r="M25" s="62"/>
+      <c r="F25" s="61"/>
+      <c r="G25" s="62"/>
+      <c r="H25" s="62"/>
+      <c r="I25" s="62"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="62"/>
+      <c r="L25" s="62"/>
+      <c r="M25" s="63"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
     </row>
     <row r="26" spans="1:15" ht="21.75" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="60" t="s">
         <v>54</v>
       </c>
       <c r="C26" s="44"/>
       <c r="D26" s="44"/>
       <c r="E26" s="10"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
-      <c r="I26" s="61"/>
-      <c r="J26" s="61"/>
-      <c r="K26" s="61"/>
-      <c r="L26" s="61"/>
-      <c r="M26" s="62"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="62"/>
+      <c r="H26" s="62"/>
+      <c r="I26" s="62"/>
+      <c r="J26" s="62"/>
+      <c r="K26" s="62"/>
+      <c r="L26" s="62"/>
+      <c r="M26" s="63"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
     </row>
@@ -8794,7 +8794,7 @@
     </row>
     <row r="29" spans="1:15" ht="19.5" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="70" t="str">
+      <c r="B29" s="74" t="str">
         <f>IF(OR(F21="",F22="",F23=""),"Ready to save — fill in the form above first","Ready to save")</f>
         <v>Ready to save — fill in the form above first</v>
       </c>
@@ -8814,7 +8814,7 @@
     </row>
     <row r="30" spans="1:15" ht="33.75" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="72" t="s">
+      <c r="B30" s="73" t="s">
         <v>77</v>
       </c>
       <c r="C30" s="44"/>
@@ -8927,26 +8927,26 @@
   </sheetData>
   <sheetProtection password="ECAF" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="62">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="B20:M20"/>
-    <mergeCell ref="K13:M13"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="K16:M16"/>
+    <mergeCell ref="F25:M25"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F21:M21"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="F24:M24"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="F11:G11"/>
     <mergeCell ref="B30:M30"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="F17:G17"/>
@@ -8963,32 +8963,32 @@
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="B29:M29"/>
+    <mergeCell ref="B20:M20"/>
+    <mergeCell ref="K13:M13"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="K16:M16"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="H16:J16"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F21:M21"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="F24:M24"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F25:M25"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="H14:J14"/>
   </mergeCells>
   <conditionalFormatting sqref="K8">
     <cfRule type="expression" dxfId="34" priority="2">
@@ -9119,12 +9119,12 @@
     </row>
     <row r="2" spans="1:15" ht="39.75" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="56" t="str">
+      <c r="B2" s="46" t="str">
         <f>CurrentBusinessName</f>
         <v>Riverside Design Studio</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
         <v>0</v>
@@ -9168,7 +9168,7 @@
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>83</v>
       </c>
       <c r="C4" s="44"/>
@@ -9204,36 +9204,36 @@
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="51" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="53"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="75" t="s">
         <v>85</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
       <c r="E7" s="10"/>
-      <c r="F7" s="79" t="s">
+      <c r="F7" s="81" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="44"/>
-      <c r="H7" s="79" t="s">
+      <c r="H7" s="81" t="s">
         <v>72</v>
       </c>
       <c r="I7" s="44"/>
@@ -9242,297 +9242,297 @@
         <v>73</v>
       </c>
       <c r="L7" s="44"/>
-      <c r="M7" s="52"/>
+      <c r="M7" s="49"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="75" t="str">
+      <c r="B8" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],1),tbl_Customers[CustomerID],0)),"")</f>
         <v>Blue Harbor Cafe</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
       <c r="E8" s="10"/>
-      <c r="F8" s="76">
+      <c r="F8" s="77">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],1),"")</f>
         <v>1200</v>
       </c>
       <c r="G8" s="44"/>
-      <c r="H8" s="78">
+      <c r="H8" s="79">
         <f ca="1">IFERROR(INDEX(tbl_Invoices[DueDate],1),"")</f>
         <v>46291</v>
       </c>
       <c r="I8" s="44"/>
       <c r="J8" s="44"/>
-      <c r="K8" s="77" t="str">
+      <c r="K8" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],1)="Paid",INDEX(tbl_Invoices[Status],1)="Void",INDEX(tbl_Invoices[Status],1)="Draft"),INDEX(tbl_Invoices[Status],1),IF(INDEX(tbl_Invoices[DueDate],1)="","",IF(INDEX(tbl_Invoices[DueDate],1)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v>Overdue</v>
       </c>
       <c r="L8" s="44"/>
-      <c r="M8" s="52"/>
+      <c r="M8" s="49"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="75" t="str">
+      <c r="B9" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],2),tbl_Customers[CustomerID],0)),"")</f>
         <v>Blue Harbor Cafe</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
       <c r="E9" s="10"/>
-      <c r="F9" s="76">
+      <c r="F9" s="77">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],2),"")</f>
         <v>500</v>
       </c>
       <c r="G9" s="44"/>
-      <c r="H9" s="78">
+      <c r="H9" s="79">
         <f ca="1">IFERROR(INDEX(tbl_Invoices[DueDate],2),"")</f>
         <v>46317</v>
       </c>
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
-      <c r="K9" s="77" t="str">
+      <c r="K9" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],2)="Paid",INDEX(tbl_Invoices[Status],2)="Void",INDEX(tbl_Invoices[Status],2)="Draft"),INDEX(tbl_Invoices[Status],2),IF(INDEX(tbl_Invoices[DueDate],2)="","",IF(INDEX(tbl_Invoices[DueDate],2)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v>Sent</v>
       </c>
       <c r="L9" s="44"/>
-      <c r="M9" s="52"/>
+      <c r="M9" s="49"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="75" t="str">
+      <c r="B10" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],3),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
       <c r="E10" s="10"/>
-      <c r="F10" s="76" t="str">
+      <c r="F10" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],3),"")</f>
         <v/>
       </c>
       <c r="G10" s="44"/>
-      <c r="H10" s="78" t="str">
+      <c r="H10" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],3),"")</f>
         <v/>
       </c>
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
-      <c r="K10" s="77" t="str">
+      <c r="K10" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],3)="Paid",INDEX(tbl_Invoices[Status],3)="Void",INDEX(tbl_Invoices[Status],3)="Draft"),INDEX(tbl_Invoices[Status],3),IF(INDEX(tbl_Invoices[DueDate],3)="","",IF(INDEX(tbl_Invoices[DueDate],3)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L10" s="44"/>
-      <c r="M10" s="52"/>
+      <c r="M10" s="49"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="75" t="str">
+      <c r="B11" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],4),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C11" s="44"/>
       <c r="D11" s="44"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="76" t="str">
+      <c r="F11" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],4),"")</f>
         <v/>
       </c>
       <c r="G11" s="44"/>
-      <c r="H11" s="78" t="str">
+      <c r="H11" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],4),"")</f>
         <v/>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
-      <c r="K11" s="77" t="str">
+      <c r="K11" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],4)="Paid",INDEX(tbl_Invoices[Status],4)="Void",INDEX(tbl_Invoices[Status],4)="Draft"),INDEX(tbl_Invoices[Status],4),IF(INDEX(tbl_Invoices[DueDate],4)="","",IF(INDEX(tbl_Invoices[DueDate],4)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L11" s="44"/>
-      <c r="M11" s="52"/>
+      <c r="M11" s="49"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="75" t="str">
+      <c r="B12" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],5),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C12" s="44"/>
       <c r="D12" s="44"/>
       <c r="E12" s="10"/>
-      <c r="F12" s="76" t="str">
+      <c r="F12" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],5),"")</f>
         <v/>
       </c>
       <c r="G12" s="44"/>
-      <c r="H12" s="78" t="str">
+      <c r="H12" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],5),"")</f>
         <v/>
       </c>
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
-      <c r="K12" s="77" t="str">
+      <c r="K12" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],5)="Paid",INDEX(tbl_Invoices[Status],5)="Void",INDEX(tbl_Invoices[Status],5)="Draft"),INDEX(tbl_Invoices[Status],5),IF(INDEX(tbl_Invoices[DueDate],5)="","",IF(INDEX(tbl_Invoices[DueDate],5)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L12" s="44"/>
-      <c r="M12" s="52"/>
+      <c r="M12" s="49"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="75" t="str">
+      <c r="B13" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],6),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C13" s="44"/>
       <c r="D13" s="44"/>
       <c r="E13" s="10"/>
-      <c r="F13" s="76" t="str">
+      <c r="F13" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],6),"")</f>
         <v/>
       </c>
       <c r="G13" s="44"/>
-      <c r="H13" s="78" t="str">
+      <c r="H13" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],6),"")</f>
         <v/>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
-      <c r="K13" s="77" t="str">
+      <c r="K13" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],6)="Paid",INDEX(tbl_Invoices[Status],6)="Void",INDEX(tbl_Invoices[Status],6)="Draft"),INDEX(tbl_Invoices[Status],6),IF(INDEX(tbl_Invoices[DueDate],6)="","",IF(INDEX(tbl_Invoices[DueDate],6)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L13" s="44"/>
-      <c r="M13" s="52"/>
+      <c r="M13" s="49"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1">
       <c r="A14" s="1"/>
-      <c r="B14" s="75" t="str">
+      <c r="B14" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],7),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C14" s="44"/>
       <c r="D14" s="44"/>
       <c r="E14" s="10"/>
-      <c r="F14" s="76" t="str">
+      <c r="F14" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],7),"")</f>
         <v/>
       </c>
       <c r="G14" s="44"/>
-      <c r="H14" s="78" t="str">
+      <c r="H14" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],7),"")</f>
         <v/>
       </c>
       <c r="I14" s="44"/>
       <c r="J14" s="44"/>
-      <c r="K14" s="77" t="str">
+      <c r="K14" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],7)="Paid",INDEX(tbl_Invoices[Status],7)="Void",INDEX(tbl_Invoices[Status],7)="Draft"),INDEX(tbl_Invoices[Status],7),IF(INDEX(tbl_Invoices[DueDate],7)="","",IF(INDEX(tbl_Invoices[DueDate],7)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L14" s="44"/>
-      <c r="M14" s="52"/>
+      <c r="M14" s="49"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="75" t="str">
+      <c r="B15" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],8),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C15" s="44"/>
       <c r="D15" s="44"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="76" t="str">
+      <c r="F15" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],8),"")</f>
         <v/>
       </c>
       <c r="G15" s="44"/>
-      <c r="H15" s="78" t="str">
+      <c r="H15" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],8),"")</f>
         <v/>
       </c>
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
-      <c r="K15" s="77" t="str">
+      <c r="K15" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],8)="Paid",INDEX(tbl_Invoices[Status],8)="Void",INDEX(tbl_Invoices[Status],8)="Draft"),INDEX(tbl_Invoices[Status],8),IF(INDEX(tbl_Invoices[DueDate],8)="","",IF(INDEX(tbl_Invoices[DueDate],8)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L15" s="44"/>
-      <c r="M15" s="52"/>
+      <c r="M15" s="49"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="75" t="str">
+      <c r="B16" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],9),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="44"/>
       <c r="D16" s="44"/>
       <c r="E16" s="10"/>
-      <c r="F16" s="76" t="str">
+      <c r="F16" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],9),"")</f>
         <v/>
       </c>
       <c r="G16" s="44"/>
-      <c r="H16" s="78" t="str">
+      <c r="H16" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],9),"")</f>
         <v/>
       </c>
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
-      <c r="K16" s="77" t="str">
+      <c r="K16" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],9)="Paid",INDEX(tbl_Invoices[Status],9)="Void",INDEX(tbl_Invoices[Status],9)="Draft"),INDEX(tbl_Invoices[Status],9),IF(INDEX(tbl_Invoices[DueDate],9)="","",IF(INDEX(tbl_Invoices[DueDate],9)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L16" s="44"/>
-      <c r="M16" s="52"/>
+      <c r="M16" s="49"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" ht="18" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="75" t="str">
+      <c r="B17" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Customers[CustomerName],MATCH(INDEX(tbl_Invoices[CustomerID],10),tbl_Customers[CustomerID],0)),"")</f>
         <v/>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="76" t="str">
+      <c r="F17" s="77" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[Amount],10),"")</f>
         <v/>
       </c>
       <c r="G17" s="44"/>
-      <c r="H17" s="78" t="str">
+      <c r="H17" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Invoices[DueDate],10),"")</f>
         <v/>
       </c>
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
-      <c r="K17" s="77" t="str">
+      <c r="K17" s="78" t="str">
         <f ca="1">IFERROR(IF(OR(INDEX(tbl_Invoices[Status],10)="Paid",INDEX(tbl_Invoices[Status],10)="Void",INDEX(tbl_Invoices[Status],10)="Draft"),INDEX(tbl_Invoices[Status],10),IF(INDEX(tbl_Invoices[DueDate],10)="","",IF(INDEX(tbl_Invoices[DueDate],10)&lt;TODAY(),"Overdue","Sent"))),"")</f>
         <v/>
       </c>
       <c r="L17" s="44"/>
-      <c r="M17" s="52"/>
+      <c r="M17" s="49"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
@@ -9572,96 +9572,96 @@
     </row>
     <row r="20" spans="1:15" ht="19.5" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48"/>
-      <c r="L20" s="48"/>
-      <c r="M20" s="49"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="52"/>
+      <c r="J20" s="52"/>
+      <c r="K20" s="52"/>
+      <c r="L20" s="52"/>
+      <c r="M20" s="53"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
     <row r="21" spans="1:15" ht="21.75" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="60" t="s">
         <v>85</v>
       </c>
       <c r="C21" s="44"/>
       <c r="D21" s="44"/>
       <c r="E21" s="10"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61"/>
-      <c r="I21" s="61"/>
-      <c r="J21" s="61"/>
-      <c r="K21" s="61"/>
-      <c r="L21" s="61"/>
-      <c r="M21" s="62"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="62"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
+      <c r="M21" s="63"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
     </row>
     <row r="22" spans="1:15" ht="21.75" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="60" t="s">
         <v>47</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="44"/>
       <c r="E22" s="10"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
-      <c r="I22" s="61"/>
-      <c r="J22" s="61"/>
-      <c r="K22" s="61"/>
-      <c r="L22" s="61"/>
-      <c r="M22" s="62"/>
+      <c r="F22" s="71"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="62"/>
+      <c r="J22" s="62"/>
+      <c r="K22" s="62"/>
+      <c r="L22" s="62"/>
+      <c r="M22" s="63"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="21.75" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="60" t="s">
         <v>72</v>
       </c>
       <c r="C23" s="44"/>
       <c r="D23" s="44"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
-      <c r="M23" s="62"/>
+      <c r="F23" s="72"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="62"/>
+      <c r="L23" s="62"/>
+      <c r="M23" s="63"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="21.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="67" t="s">
+      <c r="B24" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="57"/>
-      <c r="D24" s="57"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
       <c r="E24" s="2"/>
-      <c r="F24" s="63"/>
-      <c r="G24" s="64"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
-      <c r="L24" s="64"/>
-      <c r="M24" s="65"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
+      <c r="L24" s="67"/>
+      <c r="M24" s="68"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
     </row>
@@ -9701,7 +9701,7 @@
     </row>
     <row r="27" spans="1:15" ht="19.5" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="70" t="str">
+      <c r="B27" s="74" t="str">
         <f>IF(OR(F21="",F22="",F23=""),"Ready to save — fill in the form above first","Ready to save")</f>
         <v>Ready to save — fill in the form above first</v>
       </c>
@@ -9721,7 +9721,7 @@
     </row>
     <row r="28" spans="1:15" ht="33.75" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="72" t="s">
+      <c r="B28" s="73" t="s">
         <v>87</v>
       </c>
       <c r="C28" s="44"/>
@@ -9831,26 +9831,20 @@
   </sheetData>
   <sheetProtection password="ECAF" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="58">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="B20:M20"/>
-    <mergeCell ref="K13:M13"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="K16:M16"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="B28:M28"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F21:M21"/>
@@ -9866,29 +9860,35 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B27:M27"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="B20:M20"/>
+    <mergeCell ref="K13:M13"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="K16:M16"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="H16:J16"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="H13:J13"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="H12:J12"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K9:M9"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="F7:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="K8">
     <cfRule type="expression" dxfId="21" priority="2">
@@ -10011,12 +10011,12 @@
     </row>
     <row r="2" spans="1:15" ht="39.75" customHeight="1">
       <c r="A2" s="2"/>
-      <c r="B2" s="56" t="str">
+      <c r="B2" s="46" t="str">
         <f>CurrentBusinessName</f>
         <v>Riverside Design Studio</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
         <v>0</v>
@@ -10060,7 +10060,7 @@
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="43" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="44"/>
@@ -10096,36 +10096,36 @@
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
-      <c r="L6" s="48"/>
-      <c r="M6" s="49"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="53"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="75" t="s">
         <v>92</v>
       </c>
       <c r="C7" s="44"/>
       <c r="D7" s="44"/>
       <c r="E7" s="10"/>
-      <c r="F7" s="79" t="s">
+      <c r="F7" s="81" t="s">
         <v>93</v>
       </c>
       <c r="G7" s="44"/>
-      <c r="H7" s="79" t="s">
+      <c r="H7" s="81" t="s">
         <v>94</v>
       </c>
       <c r="I7" s="44"/>
@@ -10134,13 +10134,13 @@
         <v>73</v>
       </c>
       <c r="L7" s="44"/>
-      <c r="M7" s="52"/>
+      <c r="M7" s="49"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="75" t="str">
+      <c r="B8" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],1),"")</f>
         <v>Emergency Fund</v>
       </c>
@@ -10152,24 +10152,24 @@
         <v>$5,580 of $9,000 (62%)</v>
       </c>
       <c r="G8" s="44"/>
-      <c r="H8" s="78">
+      <c r="H8" s="79">
         <f ca="1">IFERROR(INDEX(tbl_Goals[TargetDate],1),"")</f>
         <v>46387</v>
       </c>
       <c r="I8" s="44"/>
       <c r="J8" s="44"/>
-      <c r="K8" s="77" t="str">
+      <c r="K8" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],1),"")</f>
         <v>Active</v>
       </c>
       <c r="L8" s="44"/>
-      <c r="M8" s="52"/>
+      <c r="M8" s="49"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="75" t="str">
+      <c r="B9" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],2),"")</f>
         <v/>
       </c>
@@ -10181,24 +10181,24 @@
         <v/>
       </c>
       <c r="G9" s="44"/>
-      <c r="H9" s="78" t="str">
+      <c r="H9" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Goals[TargetDate],2),"")</f>
         <v/>
       </c>
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
-      <c r="K9" s="77" t="str">
+      <c r="K9" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],2),"")</f>
         <v/>
       </c>
       <c r="L9" s="44"/>
-      <c r="M9" s="52"/>
+      <c r="M9" s="49"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="75" t="str">
+      <c r="B10" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],3),"")</f>
         <v/>
       </c>
@@ -10210,24 +10210,24 @@
         <v/>
       </c>
       <c r="G10" s="44"/>
-      <c r="H10" s="78" t="str">
+      <c r="H10" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Goals[TargetDate],3),"")</f>
         <v/>
       </c>
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
-      <c r="K10" s="77" t="str">
+      <c r="K10" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],3),"")</f>
         <v/>
       </c>
       <c r="L10" s="44"/>
-      <c r="M10" s="52"/>
+      <c r="M10" s="49"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="75" t="str">
+      <c r="B11" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],4),"")</f>
         <v/>
       </c>
@@ -10239,24 +10239,24 @@
         <v/>
       </c>
       <c r="G11" s="44"/>
-      <c r="H11" s="78" t="str">
+      <c r="H11" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Goals[TargetDate],4),"")</f>
         <v/>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
-      <c r="K11" s="77" t="str">
+      <c r="K11" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],4),"")</f>
         <v/>
       </c>
       <c r="L11" s="44"/>
-      <c r="M11" s="52"/>
+      <c r="M11" s="49"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="75" t="str">
+      <c r="B12" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],5),"")</f>
         <v/>
       </c>
@@ -10268,24 +10268,24 @@
         <v/>
       </c>
       <c r="G12" s="44"/>
-      <c r="H12" s="78" t="str">
+      <c r="H12" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Goals[TargetDate],5),"")</f>
         <v/>
       </c>
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
-      <c r="K12" s="77" t="str">
+      <c r="K12" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],5),"")</f>
         <v/>
       </c>
       <c r="L12" s="44"/>
-      <c r="M12" s="52"/>
+      <c r="M12" s="49"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="75" t="str">
+      <c r="B13" s="76" t="str">
         <f>IFERROR(INDEX(tbl_Goals[GoalName],6),"")</f>
         <v/>
       </c>
@@ -10297,18 +10297,18 @@
         <v/>
       </c>
       <c r="G13" s="44"/>
-      <c r="H13" s="78" t="str">
+      <c r="H13" s="79" t="str">
         <f>IFERROR(INDEX(tbl_Goals[TargetDate],6),"")</f>
         <v/>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
-      <c r="K13" s="77" t="str">
+      <c r="K13" s="78" t="str">
         <f>IFERROR(INDEX(tbl_Goals[Status],6),"")</f>
         <v/>
       </c>
       <c r="L13" s="44"/>
-      <c r="M13" s="52"/>
+      <c r="M13" s="49"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
@@ -10348,96 +10348,96 @@
     </row>
     <row r="16" spans="1:15" ht="19.5" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="47" t="s">
+      <c r="B16" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="48"/>
-      <c r="H16" s="48"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="48"/>
-      <c r="K16" s="48"/>
-      <c r="L16" s="48"/>
-      <c r="M16" s="49"/>
+      <c r="C16" s="52"/>
+      <c r="D16" s="52"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="52"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
+      <c r="M16" s="53"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" ht="21.75" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="60" t="s">
         <v>96</v>
       </c>
       <c r="C17" s="44"/>
       <c r="D17" s="44"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="62"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="62"/>
+      <c r="J17" s="62"/>
+      <c r="K17" s="62"/>
+      <c r="L17" s="62"/>
+      <c r="M17" s="63"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="21.75" customHeight="1">
       <c r="A18" s="1"/>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="60" t="s">
         <v>97</v>
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="44"/>
       <c r="E18" s="10"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="61"/>
-      <c r="K18" s="61"/>
-      <c r="L18" s="61"/>
-      <c r="M18" s="62"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
+      <c r="I18" s="62"/>
+      <c r="J18" s="62"/>
+      <c r="K18" s="62"/>
+      <c r="L18" s="62"/>
+      <c r="M18" s="63"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
     </row>
     <row r="19" spans="1:15" ht="21.75" customHeight="1">
       <c r="A19" s="1"/>
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="60" t="s">
         <v>98</v>
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="44"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="61"/>
-      <c r="H19" s="61"/>
-      <c r="I19" s="61"/>
-      <c r="J19" s="61"/>
-      <c r="K19" s="61"/>
-      <c r="L19" s="61"/>
-      <c r="M19" s="62"/>
+      <c r="F19" s="71"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="62"/>
+      <c r="J19" s="62"/>
+      <c r="K19" s="62"/>
+      <c r="L19" s="62"/>
+      <c r="M19" s="63"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="21.75" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="67" t="s">
+      <c r="B20" s="64" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
       <c r="E20" s="2"/>
       <c r="F20" s="83"/>
-      <c r="G20" s="64"/>
-      <c r="H20" s="64"/>
-      <c r="I20" s="64"/>
-      <c r="J20" s="64"/>
-      <c r="K20" s="64"/>
-      <c r="L20" s="64"/>
-      <c r="M20" s="65"/>
+      <c r="G20" s="67"/>
+      <c r="H20" s="67"/>
+      <c r="I20" s="67"/>
+      <c r="J20" s="67"/>
+      <c r="K20" s="67"/>
+      <c r="L20" s="67"/>
+      <c r="M20" s="68"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
@@ -10477,7 +10477,7 @@
     </row>
     <row r="23" spans="1:15" ht="19.5" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="70" t="str">
+      <c r="B23" s="74" t="str">
         <f>IF(OR(F17="",F18="",F19=""),"Ready to save — fill in the form above first","Ready to save")</f>
         <v>Ready to save — fill in the form above first</v>
       </c>
@@ -10497,7 +10497,7 @@
     </row>
     <row r="24" spans="1:15" ht="33.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="72" t="s">
+      <c r="B24" s="73" t="s">
         <v>100</v>
       </c>
       <c r="C24" s="44"/>
@@ -10610,6 +10610,32 @@
   </sheetData>
   <sheetProtection password="ECAF" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="42">
+    <mergeCell ref="B23:M23"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="F20:M20"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F19:M19"/>
+    <mergeCell ref="B24:M24"/>
+    <mergeCell ref="F17:M17"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="K13:M13"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="K8:M8"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="F18:M18"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B4:M4"/>
     <mergeCell ref="F9:G9"/>
@@ -10619,39 +10645,13 @@
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B6:M6"/>
-    <mergeCell ref="B24:M24"/>
-    <mergeCell ref="F17:M17"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="K13:M13"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="F13:G13"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B18:D18"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="F18:M18"/>
     <mergeCell ref="K7:M7"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B23:M23"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="F20:M20"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="F11:G11"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F19:M19"/>
   </mergeCells>
   <conditionalFormatting sqref="K8">
     <cfRule type="expression" dxfId="8" priority="2">

</xml_diff>